<commit_message>
#55 Reading List: updated to 2026-08-23.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99155C18-56D5-4CFF-AA34-378925775D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67389D4-5E2E-4ACA-8146-2ECB5E1FB3BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1140" yWindow="435" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="765" yWindow="690" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed2016" sheetId="16" state="hidden" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5875" uniqueCount="1245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5947" uniqueCount="1261">
   <si>
     <t>Format</t>
   </si>
@@ -3781,6 +3781,54 @@
   </si>
   <si>
     <t>The Security Metrics Workbook</t>
+  </si>
+  <si>
+    <t>Agentic AI Playbook</t>
+  </si>
+  <si>
+    <t>2026-08-02</t>
+  </si>
+  <si>
+    <t>Useful. A comprehensive introduction to the topic, clearly written and structured.</t>
+  </si>
+  <si>
+    <t>Agentic Coding with Claude Code</t>
+  </si>
+  <si>
+    <t>2026-08-07</t>
+  </si>
+  <si>
+    <t>Useful. A quite valid introductory book about Claude Code and agentic architecture.</t>
+  </si>
+  <si>
+    <t>Building CLI Applications With C# and .NET</t>
+  </si>
+  <si>
+    <t>Useful. Comprehensive book for beginners. The author uses a lot of smileys, which I find unprofessional.</t>
+  </si>
+  <si>
+    <t>AI Agents In Action</t>
+  </si>
+  <si>
+    <t>2026-08-14</t>
+  </si>
+  <si>
+    <t>Useless. The book doesn't contain much actionable knowledge but it roams around the topic offering code examples and diagrams of doubtful usefulness. The book lacks of an easy-to-scan layout (no bold faces). From Manning I do expect more quality.</t>
+  </si>
+  <si>
+    <t>Building Applications with AI Agents</t>
+  </si>
+  <si>
+    <t>From Zero To Pro With Claude AI</t>
+  </si>
+  <si>
+    <t>2026-08-23</t>
+  </si>
+  <si>
+    <t>Useful. Very dense and well-written book. It contains knowledge I didn't find elsewhere and it doesn't repeat itself. It lacks of bold fonts.</t>
+  </si>
+  <si>
+    <t>Useless. A book for beginners written in a very repetitive and redundant style. Some content could be communicated in half amount of pages wit hno loss of information.</t>
   </si>
 </sst>
 </file>
@@ -3926,7 +3974,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4052,7 +4100,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11519,7 +11566,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:U400"/>
+  <dimension ref="A1:U406"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -37472,11 +37519,11 @@
         <v>1216</v>
       </c>
       <c r="H382" s="9">
-        <f t="shared" ref="H382:H389" si="216">YEAR(G382)</f>
+        <f t="shared" ref="H382:H393" si="216">YEAR(G382)</f>
         <v>2026</v>
       </c>
       <c r="I382" s="9">
-        <f t="shared" ref="I382:I389" si="217">MONTH(G382)</f>
+        <f t="shared" ref="I382:I391" si="217">MONTH(G382)</f>
         <v>5</v>
       </c>
       <c r="J382" s="9" t="s">
@@ -37669,7 +37716,7 @@
       <c r="E385" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F385" s="44">
+      <c r="F385" s="14">
         <v>252</v>
       </c>
       <c r="G385" s="9" t="s">
@@ -37692,16 +37739,16 @@
       <c r="L385" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M385" s="44">
+      <c r="M385" s="14">
         <v>3</v>
       </c>
-      <c r="N385" s="44">
+      <c r="N385" s="14">
         <v>36.99</v>
       </c>
       <c r="O385" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P385" s="45" t="s">
+      <c r="P385" s="22" t="s">
         <v>1235</v>
       </c>
       <c r="Q385" s="9" t="s">
@@ -37737,7 +37784,7 @@
       <c r="E386" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F386" s="44">
+      <c r="F386" s="14">
         <v>152</v>
       </c>
       <c r="G386" s="9" t="s">
@@ -37760,7 +37807,7 @@
       <c r="L386" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M386" s="44">
+      <c r="M386" s="14">
         <v>3</v>
       </c>
       <c r="N386" s="35">
@@ -37805,7 +37852,7 @@
       <c r="E387" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F387" s="44">
+      <c r="F387" s="14">
         <v>137</v>
       </c>
       <c r="G387" s="9" t="s">
@@ -37828,10 +37875,10 @@
       <c r="L387" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M387" s="44">
+      <c r="M387" s="14">
         <v>3</v>
       </c>
-      <c r="N387" s="44">
+      <c r="N387" s="14">
         <v>9.99</v>
       </c>
       <c r="O387" s="9" t="s">
@@ -37873,7 +37920,7 @@
       <c r="E388" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F388" s="44">
+      <c r="F388" s="14">
         <v>356</v>
       </c>
       <c r="G388" s="9" t="s">
@@ -37896,16 +37943,16 @@
       <c r="L388" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M388" s="44">
+      <c r="M388" s="14">
         <v>2</v>
       </c>
-      <c r="N388" s="44">
+      <c r="N388" s="14">
         <v>54.99</v>
       </c>
       <c r="O388" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P388" s="45" t="s">
+      <c r="P388" s="22" t="s">
         <v>1243</v>
       </c>
       <c r="Q388" s="9" t="s">
@@ -37929,7 +37976,7 @@
       <c r="A389" s="7" t="s">
         <v>1244</v>
       </c>
-      <c r="B389" s="44">
+      <c r="B389" s="14">
         <v>2026</v>
       </c>
       <c r="C389" s="9" t="s">
@@ -37941,7 +37988,7 @@
       <c r="E389" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F389" s="44">
+      <c r="F389" s="14">
         <v>122</v>
       </c>
       <c r="G389" s="9" t="s">
@@ -37964,16 +38011,16 @@
       <c r="L389" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M389" s="44">
+      <c r="M389" s="14">
         <v>3</v>
       </c>
-      <c r="N389" s="44">
+      <c r="N389" s="14">
         <v>19.989999999999998</v>
       </c>
       <c r="O389" s="9" t="s">
         <v>632</v>
       </c>
-      <c r="P389" s="45" t="s">
+      <c r="P389" s="22" t="s">
         <v>1243</v>
       </c>
       <c r="Q389" s="9" t="s">
@@ -37983,7 +38030,7 @@
         <v>153</v>
       </c>
       <c r="S389" s="14">
-        <f t="shared" ref="S389" si="219">LEN(P389)</f>
+        <f t="shared" ref="S389:S395" si="219">LEN(P389)</f>
         <v>30</v>
       </c>
       <c r="T389" s="14">
@@ -37994,142 +38041,412 @@
       </c>
     </row>
     <row r="390" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A390" s="7"/>
-      <c r="B390" s="9"/>
-      <c r="C390" s="9"/>
-      <c r="D390" s="9"/>
-      <c r="E390" s="9"/>
-      <c r="F390" s="9"/>
-      <c r="G390" s="9"/>
-      <c r="H390" s="9"/>
-      <c r="I390" s="9"/>
-      <c r="J390" s="9"/>
-      <c r="K390" s="9"/>
-      <c r="L390" s="9"/>
-      <c r="M390" s="9"/>
-      <c r="N390" s="9"/>
-      <c r="O390" s="9"/>
-      <c r="P390" s="12"/>
-      <c r="Q390" s="9"/>
-      <c r="R390" s="9"/>
-      <c r="S390" s="14"/>
-      <c r="T390" s="9"/>
-      <c r="U390" s="14"/>
+      <c r="A390" s="7" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B390" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C390" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D390" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E390" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F390" s="44">
+        <v>222</v>
+      </c>
+      <c r="G390" s="9" t="s">
+        <v>1246</v>
+      </c>
+      <c r="H390" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I390" s="9">
+        <f t="shared" si="217"/>
+        <v>8</v>
+      </c>
+      <c r="J390" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K390" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L390" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M390" s="44">
+        <v>3</v>
+      </c>
+      <c r="N390" s="44">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="O390" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P390" s="12" t="s">
+        <v>1247</v>
+      </c>
+      <c r="Q390" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R390" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S390" s="14">
+        <f t="shared" si="219"/>
+        <v>82</v>
+      </c>
+      <c r="T390" s="14">
+        <v>0</v>
+      </c>
+      <c r="U390" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="391" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A391" s="7"/>
-      <c r="B391" s="9"/>
-      <c r="C391" s="9"/>
-      <c r="D391" s="9"/>
-      <c r="E391" s="9"/>
-      <c r="F391" s="9"/>
-      <c r="G391" s="9"/>
-      <c r="H391" s="9"/>
-      <c r="I391" s="9"/>
-      <c r="J391" s="9"/>
-      <c r="K391" s="9"/>
-      <c r="L391" s="9"/>
-      <c r="M391" s="9"/>
-      <c r="N391" s="9"/>
-      <c r="O391" s="9"/>
-      <c r="P391" s="12"/>
-      <c r="Q391" s="9"/>
-      <c r="R391" s="9"/>
-      <c r="S391" s="14"/>
-      <c r="T391" s="9"/>
-      <c r="U391" s="14"/>
+      <c r="A391" s="7" t="s">
+        <v>1248</v>
+      </c>
+      <c r="B391" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C391" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D391" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E391" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F391" s="44">
+        <v>377</v>
+      </c>
+      <c r="G391" s="9" t="s">
+        <v>1249</v>
+      </c>
+      <c r="H391" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I391" s="9">
+        <f t="shared" si="217"/>
+        <v>8</v>
+      </c>
+      <c r="J391" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K391" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L391" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M391" s="44">
+        <v>3</v>
+      </c>
+      <c r="N391" s="44">
+        <v>44.99</v>
+      </c>
+      <c r="O391" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P391" s="12" t="s">
+        <v>1250</v>
+      </c>
+      <c r="Q391" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R391" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S391" s="14">
+        <f t="shared" si="219"/>
+        <v>83</v>
+      </c>
+      <c r="T391" s="14">
+        <v>0</v>
+      </c>
+      <c r="U391" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="392" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A392" s="7"/>
-      <c r="B392" s="9"/>
-      <c r="C392" s="9"/>
-      <c r="D392" s="9"/>
-      <c r="E392" s="9"/>
-      <c r="F392" s="9"/>
-      <c r="G392" s="9"/>
-      <c r="H392" s="9"/>
-      <c r="I392" s="9"/>
-      <c r="J392" s="9"/>
-      <c r="K392" s="9"/>
-      <c r="L392" s="9"/>
-      <c r="M392" s="9"/>
-      <c r="N392" s="9"/>
-      <c r="O392" s="9"/>
-      <c r="P392" s="12"/>
-      <c r="Q392" s="9"/>
-      <c r="R392" s="9"/>
-      <c r="S392" s="14"/>
-      <c r="T392" s="9"/>
-      <c r="U392" s="14"/>
+      <c r="A392" s="7" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B392" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C392" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D392" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E392" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F392" s="44">
+        <v>293</v>
+      </c>
+      <c r="G392" s="9" t="s">
+        <v>1249</v>
+      </c>
+      <c r="H392" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I392" s="9">
+        <f t="shared" ref="I392" si="220">MONTH(G392)</f>
+        <v>8</v>
+      </c>
+      <c r="J392" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K392" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L392" s="9" t="s">
+        <v>341</v>
+      </c>
+      <c r="M392" s="44">
+        <v>2</v>
+      </c>
+      <c r="N392" s="44">
+        <v>41.99</v>
+      </c>
+      <c r="O392" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P392" s="12" t="s">
+        <v>1252</v>
+      </c>
+      <c r="Q392" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="R392" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S392" s="14">
+        <f t="shared" si="219"/>
+        <v>104</v>
+      </c>
+      <c r="T392" s="14">
+        <v>0</v>
+      </c>
+      <c r="U392" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="393" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A393" s="7"/>
-      <c r="B393" s="9"/>
-      <c r="C393" s="9"/>
-      <c r="D393" s="9"/>
-      <c r="E393" s="9"/>
-      <c r="F393" s="9"/>
-      <c r="G393" s="9"/>
-      <c r="H393" s="9"/>
-      <c r="I393" s="9"/>
-      <c r="J393" s="9"/>
-      <c r="K393" s="9"/>
-      <c r="L393" s="9"/>
-      <c r="M393" s="9"/>
-      <c r="N393" s="9"/>
-      <c r="O393" s="9"/>
-      <c r="P393" s="12"/>
-      <c r="Q393" s="9"/>
-      <c r="R393" s="9"/>
-      <c r="S393" s="14"/>
-      <c r="T393" s="9"/>
-      <c r="U393" s="14"/>
+      <c r="A393" s="7" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B393" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C393" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D393" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E393" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F393" s="44">
+        <v>346</v>
+      </c>
+      <c r="G393" s="9" t="s">
+        <v>1254</v>
+      </c>
+      <c r="H393" s="9">
+        <f t="shared" si="216"/>
+        <v>2026</v>
+      </c>
+      <c r="I393" s="9">
+        <f t="shared" ref="I393" si="221">MONTH(G393)</f>
+        <v>8</v>
+      </c>
+      <c r="J393" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K393" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L393" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M393" s="44">
+        <v>1</v>
+      </c>
+      <c r="N393" s="44">
+        <v>59.99</v>
+      </c>
+      <c r="O393" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P393" s="12" t="s">
+        <v>1255</v>
+      </c>
+      <c r="Q393" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R393" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S393" s="14">
+        <f t="shared" si="219"/>
+        <v>246</v>
+      </c>
+      <c r="T393" s="14">
+        <v>0</v>
+      </c>
+      <c r="U393" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="394" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A394" s="7"/>
-      <c r="B394" s="9"/>
-      <c r="C394" s="9"/>
-      <c r="D394" s="9"/>
-      <c r="E394" s="9"/>
-      <c r="F394" s="9"/>
-      <c r="G394" s="9"/>
-      <c r="H394" s="9"/>
-      <c r="I394" s="9"/>
-      <c r="J394" s="9"/>
-      <c r="K394" s="9"/>
-      <c r="L394" s="9"/>
-      <c r="M394" s="9"/>
-      <c r="N394" s="9"/>
-      <c r="O394" s="9"/>
-      <c r="P394" s="12"/>
-      <c r="Q394" s="9"/>
-      <c r="R394" s="9"/>
-      <c r="S394" s="14"/>
-      <c r="T394" s="9"/>
-      <c r="U394" s="14"/>
+      <c r="A394" s="7" t="s">
+        <v>1256</v>
+      </c>
+      <c r="B394" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C394" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D394" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E394" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F394" s="44">
+        <v>355</v>
+      </c>
+      <c r="G394" s="9" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H394" s="9">
+        <f t="shared" ref="H394:H395" si="222">YEAR(G394)</f>
+        <v>2026</v>
+      </c>
+      <c r="I394" s="9">
+        <f t="shared" ref="I394:I395" si="223">MONTH(G394)</f>
+        <v>8</v>
+      </c>
+      <c r="J394" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K394" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L394" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M394" s="44">
+        <v>4</v>
+      </c>
+      <c r="N394" s="44">
+        <v>79.989999999999995</v>
+      </c>
+      <c r="O394" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P394" s="12" t="s">
+        <v>1259</v>
+      </c>
+      <c r="Q394" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R394" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S394" s="14">
+        <f t="shared" si="219"/>
+        <v>141</v>
+      </c>
+      <c r="T394" s="14">
+        <v>0</v>
+      </c>
+      <c r="U394" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="395" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A395" s="7"/>
-      <c r="B395" s="9"/>
-      <c r="C395" s="9"/>
-      <c r="D395" s="9"/>
-      <c r="E395" s="9"/>
-      <c r="F395" s="9"/>
-      <c r="G395" s="9"/>
-      <c r="H395" s="9"/>
-      <c r="I395" s="9"/>
-      <c r="J395" s="9"/>
-      <c r="K395" s="9"/>
-      <c r="L395" s="9"/>
-      <c r="M395" s="9"/>
-      <c r="N395" s="9"/>
-      <c r="O395" s="9"/>
-      <c r="P395" s="12"/>
-      <c r="Q395" s="9"/>
-      <c r="R395" s="9"/>
-      <c r="S395" s="14"/>
-      <c r="T395" s="9"/>
-      <c r="U395" s="14"/>
+      <c r="A395" s="7" t="s">
+        <v>1257</v>
+      </c>
+      <c r="B395" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C395" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D395" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E395" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F395" s="44">
+        <v>317</v>
+      </c>
+      <c r="G395" s="9" t="s">
+        <v>1258</v>
+      </c>
+      <c r="H395" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I395" s="9">
+        <f t="shared" si="223"/>
+        <v>8</v>
+      </c>
+      <c r="J395" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K395" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L395" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M395" s="44">
+        <v>1</v>
+      </c>
+      <c r="N395" s="44">
+        <v>29.99</v>
+      </c>
+      <c r="O395" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P395" s="12" t="s">
+        <v>1260</v>
+      </c>
+      <c r="Q395" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R395" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S395" s="14">
+        <f t="shared" si="219"/>
+        <v>167</v>
+      </c>
+      <c r="T395" s="14">
+        <v>0</v>
+      </c>
+      <c r="U395" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="396" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A396" s="7"/>
@@ -38245,6 +38562,144 @@
       <c r="S400" s="14"/>
       <c r="T400" s="9"/>
       <c r="U400" s="14"/>
+    </row>
+    <row r="401" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A401" s="9"/>
+      <c r="B401" s="9"/>
+      <c r="C401" s="9"/>
+      <c r="D401" s="9"/>
+      <c r="E401" s="9"/>
+      <c r="F401" s="9"/>
+      <c r="G401" s="9"/>
+      <c r="H401" s="9"/>
+      <c r="I401" s="9"/>
+      <c r="J401" s="9"/>
+      <c r="K401" s="9"/>
+      <c r="L401" s="9"/>
+      <c r="M401" s="9"/>
+      <c r="N401" s="9"/>
+      <c r="O401" s="9"/>
+      <c r="P401" s="9"/>
+      <c r="Q401" s="9"/>
+      <c r="R401" s="9"/>
+      <c r="S401" s="14"/>
+      <c r="T401" s="9"/>
+      <c r="U401" s="14"/>
+    </row>
+    <row r="402" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A402" s="9"/>
+      <c r="B402" s="9"/>
+      <c r="C402" s="9"/>
+      <c r="D402" s="9"/>
+      <c r="E402" s="9"/>
+      <c r="F402" s="9"/>
+      <c r="G402" s="9"/>
+      <c r="H402" s="9"/>
+      <c r="I402" s="9"/>
+      <c r="J402" s="9"/>
+      <c r="K402" s="9"/>
+      <c r="L402" s="9"/>
+      <c r="M402" s="9"/>
+      <c r="N402" s="9"/>
+      <c r="O402" s="9"/>
+      <c r="P402" s="9"/>
+      <c r="Q402" s="9"/>
+      <c r="R402" s="9"/>
+      <c r="S402" s="14"/>
+      <c r="T402" s="9"/>
+      <c r="U402" s="14"/>
+    </row>
+    <row r="403" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A403" s="9"/>
+      <c r="B403" s="9"/>
+      <c r="C403" s="9"/>
+      <c r="D403" s="9"/>
+      <c r="E403" s="9"/>
+      <c r="F403" s="9"/>
+      <c r="G403" s="9"/>
+      <c r="H403" s="9"/>
+      <c r="I403" s="9"/>
+      <c r="J403" s="9"/>
+      <c r="K403" s="9"/>
+      <c r="L403" s="9"/>
+      <c r="M403" s="9"/>
+      <c r="N403" s="9"/>
+      <c r="O403" s="9"/>
+      <c r="P403" s="9"/>
+      <c r="Q403" s="9"/>
+      <c r="R403" s="9"/>
+      <c r="S403" s="14"/>
+      <c r="T403" s="9"/>
+      <c r="U403" s="14"/>
+    </row>
+    <row r="404" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A404" s="9"/>
+      <c r="B404" s="9"/>
+      <c r="C404" s="9"/>
+      <c r="D404" s="9"/>
+      <c r="E404" s="9"/>
+      <c r="F404" s="9"/>
+      <c r="G404" s="9"/>
+      <c r="H404" s="9"/>
+      <c r="I404" s="9"/>
+      <c r="J404" s="9"/>
+      <c r="K404" s="9"/>
+      <c r="L404" s="9"/>
+      <c r="M404" s="9"/>
+      <c r="N404" s="9"/>
+      <c r="O404" s="9"/>
+      <c r="P404" s="9"/>
+      <c r="Q404" s="9"/>
+      <c r="R404" s="9"/>
+      <c r="S404" s="14"/>
+      <c r="T404" s="9"/>
+      <c r="U404" s="14"/>
+    </row>
+    <row r="405" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A405" s="9"/>
+      <c r="B405" s="9"/>
+      <c r="C405" s="9"/>
+      <c r="D405" s="9"/>
+      <c r="E405" s="9"/>
+      <c r="F405" s="9"/>
+      <c r="G405" s="9"/>
+      <c r="H405" s="9"/>
+      <c r="I405" s="9"/>
+      <c r="J405" s="9"/>
+      <c r="K405" s="9"/>
+      <c r="L405" s="9"/>
+      <c r="M405" s="9"/>
+      <c r="N405" s="9"/>
+      <c r="O405" s="9"/>
+      <c r="P405" s="9"/>
+      <c r="Q405" s="9"/>
+      <c r="R405" s="9"/>
+      <c r="S405" s="14"/>
+      <c r="T405" s="9"/>
+      <c r="U405" s="14"/>
+    </row>
+    <row r="406" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A406" s="9"/>
+      <c r="B406" s="9"/>
+      <c r="C406" s="9"/>
+      <c r="D406" s="9"/>
+      <c r="E406" s="9"/>
+      <c r="F406" s="9"/>
+      <c r="G406" s="9"/>
+      <c r="H406" s="9"/>
+      <c r="I406" s="9"/>
+      <c r="J406" s="9"/>
+      <c r="K406" s="9"/>
+      <c r="L406" s="9"/>
+      <c r="M406" s="9"/>
+      <c r="N406" s="9"/>
+      <c r="O406" s="9"/>
+      <c r="P406" s="9"/>
+      <c r="Q406" s="9"/>
+      <c r="R406" s="9"/>
+      <c r="S406" s="14"/>
+      <c r="T406" s="9"/>
+      <c r="U406" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
#55 Reading List: updated to 2026-09-28.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67389D4-5E2E-4ACA-8146-2ECB5E1FB3BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE92AB3-44F7-43E6-9B25-AF6B0584C98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="765" yWindow="690" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="660" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed2016" sheetId="16" state="hidden" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5947" uniqueCount="1261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6007" uniqueCount="1274">
   <si>
     <t>Format</t>
   </si>
@@ -3829,6 +3829,45 @@
   </si>
   <si>
     <t>Useless. A book for beginners written in a very repetitive and redundant style. Some content could be communicated in half amount of pages wit hno loss of information.</t>
+  </si>
+  <si>
+    <t>Mindset</t>
+  </si>
+  <si>
+    <t>2026-09-27</t>
+  </si>
+  <si>
+    <t>Random House</t>
+  </si>
+  <si>
+    <t>Useless. Verbose and redundant, it could be summarized in 15 pages without loss of content.</t>
+  </si>
+  <si>
+    <t>TDD With Python</t>
+  </si>
+  <si>
+    <t>Useless. The code snippets are in Spanish and the author doesn't explain a way to run unit tests automatically while the developers write code, which it's the basic of TDD.</t>
+  </si>
+  <si>
+    <t>Laws of Software Engineering</t>
+  </si>
+  <si>
+    <t>Useful. Very well written, concise, easy to scan. I didn't know the 70% of these laws, therefore I assume few software engineering books talk about them.</t>
+  </si>
+  <si>
+    <t>Modern Software Engineering</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>Useless. Ok as getting started guide, but nothing new for non-beginners.</t>
+  </si>
+  <si>
+    <t>Software Design For Python Programmers</t>
+  </si>
+  <si>
+    <t>Useless. Ok as getting started guide, but nothing new for non-beginners. The book is also hyper-dense of examples, which slow down the reading.</t>
   </si>
 </sst>
 </file>
@@ -3974,7 +4013,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4095,9 +4134,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -38030,7 +38066,7 @@
         <v>153</v>
       </c>
       <c r="S389" s="14">
-        <f t="shared" ref="S389:S395" si="219">LEN(P389)</f>
+        <f t="shared" ref="S389:S400" si="219">LEN(P389)</f>
         <v>30</v>
       </c>
       <c r="T389" s="14">
@@ -38056,7 +38092,7 @@
       <c r="E390" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F390" s="44">
+      <c r="F390" s="14">
         <v>222</v>
       </c>
       <c r="G390" s="9" t="s">
@@ -38079,10 +38115,10 @@
       <c r="L390" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M390" s="44">
+      <c r="M390" s="14">
         <v>3</v>
       </c>
-      <c r="N390" s="44">
+      <c r="N390" s="14">
         <v>19.989999999999998</v>
       </c>
       <c r="O390" s="9" t="s">
@@ -38124,7 +38160,7 @@
       <c r="E391" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F391" s="44">
+      <c r="F391" s="14">
         <v>377</v>
       </c>
       <c r="G391" s="9" t="s">
@@ -38147,10 +38183,10 @@
       <c r="L391" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M391" s="44">
+      <c r="M391" s="14">
         <v>3</v>
       </c>
-      <c r="N391" s="44">
+      <c r="N391" s="14">
         <v>44.99</v>
       </c>
       <c r="O391" s="9" t="s">
@@ -38192,7 +38228,7 @@
       <c r="E392" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F392" s="44">
+      <c r="F392" s="14">
         <v>293</v>
       </c>
       <c r="G392" s="9" t="s">
@@ -38215,10 +38251,10 @@
       <c r="L392" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="M392" s="44">
+      <c r="M392" s="14">
         <v>2</v>
       </c>
-      <c r="N392" s="44">
+      <c r="N392" s="14">
         <v>41.99</v>
       </c>
       <c r="O392" s="9" t="s">
@@ -38260,7 +38296,7 @@
       <c r="E393" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F393" s="44">
+      <c r="F393" s="14">
         <v>346</v>
       </c>
       <c r="G393" s="9" t="s">
@@ -38283,10 +38319,10 @@
       <c r="L393" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="M393" s="44">
+      <c r="M393" s="14">
         <v>1</v>
       </c>
-      <c r="N393" s="44">
+      <c r="N393" s="14">
         <v>59.99</v>
       </c>
       <c r="O393" s="9" t="s">
@@ -38328,18 +38364,18 @@
       <c r="E394" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F394" s="44">
+      <c r="F394" s="14">
         <v>355</v>
       </c>
       <c r="G394" s="9" t="s">
         <v>1258</v>
       </c>
       <c r="H394" s="9">
-        <f t="shared" ref="H394:H395" si="222">YEAR(G394)</f>
+        <f t="shared" ref="H394:H400" si="222">YEAR(G394)</f>
         <v>2026</v>
       </c>
       <c r="I394" s="9">
-        <f t="shared" ref="I394:I395" si="223">MONTH(G394)</f>
+        <f t="shared" ref="I394:I396" si="223">MONTH(G394)</f>
         <v>8</v>
       </c>
       <c r="J394" s="9" t="s">
@@ -38351,10 +38387,10 @@
       <c r="L394" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="M394" s="44">
-        <v>4</v>
-      </c>
-      <c r="N394" s="44">
+      <c r="M394" s="14">
+        <v>4</v>
+      </c>
+      <c r="N394" s="14">
         <v>79.989999999999995</v>
       </c>
       <c r="O394" s="9" t="s">
@@ -38396,7 +38432,7 @@
       <c r="E395" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F395" s="44">
+      <c r="F395" s="14">
         <v>317</v>
       </c>
       <c r="G395" s="9" t="s">
@@ -38419,10 +38455,10 @@
       <c r="L395" s="9" t="s">
         <v>570</v>
       </c>
-      <c r="M395" s="44">
+      <c r="M395" s="14">
         <v>1</v>
       </c>
-      <c r="N395" s="44">
+      <c r="N395" s="14">
         <v>29.99</v>
       </c>
       <c r="O395" s="9" t="s">
@@ -38449,119 +38485,344 @@
       </c>
     </row>
     <row r="396" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A396" s="7"/>
-      <c r="B396" s="9"/>
-      <c r="C396" s="9"/>
-      <c r="D396" s="9"/>
-      <c r="E396" s="9"/>
-      <c r="F396" s="9"/>
-      <c r="G396" s="9"/>
-      <c r="H396" s="9"/>
-      <c r="I396" s="9"/>
-      <c r="J396" s="9"/>
-      <c r="K396" s="9"/>
-      <c r="L396" s="9"/>
-      <c r="M396" s="9"/>
-      <c r="N396" s="9"/>
-      <c r="O396" s="9"/>
-      <c r="P396" s="12"/>
-      <c r="Q396" s="9"/>
-      <c r="R396" s="9"/>
-      <c r="S396" s="14"/>
-      <c r="T396" s="9"/>
-      <c r="U396" s="14"/>
+      <c r="A396" s="7" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B396" s="14">
+        <v>2017</v>
+      </c>
+      <c r="C396" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D396" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E396" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F396" s="14">
+        <v>306</v>
+      </c>
+      <c r="G396" s="9" t="s">
+        <v>1262</v>
+      </c>
+      <c r="H396" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I396" s="9">
+        <f t="shared" si="223"/>
+        <v>9</v>
+      </c>
+      <c r="J396" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K396" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L396" s="9" t="s">
+        <v>1263</v>
+      </c>
+      <c r="M396" s="14">
+        <v>1</v>
+      </c>
+      <c r="N396" s="14">
+        <v>32</v>
+      </c>
+      <c r="O396" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P396" s="12" t="s">
+        <v>1264</v>
+      </c>
+      <c r="Q396" s="9" t="s">
+        <v>1187</v>
+      </c>
+      <c r="R396" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S396" s="14">
+        <f t="shared" si="219"/>
+        <v>91</v>
+      </c>
+      <c r="T396" s="14">
+        <v>0</v>
+      </c>
+      <c r="U396" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="397" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A397" s="7"/>
-      <c r="B397" s="9"/>
-      <c r="C397" s="9"/>
-      <c r="D397" s="9"/>
-      <c r="E397" s="9"/>
-      <c r="F397" s="9"/>
-      <c r="G397" s="9"/>
-      <c r="H397" s="9"/>
-      <c r="I397" s="9"/>
-      <c r="J397" s="9"/>
-      <c r="K397" s="9"/>
-      <c r="L397" s="9"/>
-      <c r="M397" s="9"/>
-      <c r="N397" s="9"/>
-      <c r="O397" s="9"/>
-      <c r="P397" s="12"/>
-      <c r="Q397" s="9"/>
-      <c r="R397" s="9"/>
-      <c r="S397" s="14"/>
-      <c r="T397" s="9"/>
-      <c r="U397" s="14"/>
+      <c r="A397" s="7" t="s">
+        <v>1265</v>
+      </c>
+      <c r="B397" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C397" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D397" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E397" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F397" s="14">
+        <v>114</v>
+      </c>
+      <c r="G397" s="9" t="s">
+        <v>1262</v>
+      </c>
+      <c r="H397" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I397" s="9">
+        <f t="shared" ref="I397:I400" si="224">MONTH(G397)</f>
+        <v>9</v>
+      </c>
+      <c r="J397" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K397" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L397" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M397" s="14">
+        <v>1</v>
+      </c>
+      <c r="N397" s="35">
+        <v>0</v>
+      </c>
+      <c r="O397" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P397" s="22" t="s">
+        <v>1266</v>
+      </c>
+      <c r="Q397" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="R397" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S397" s="14">
+        <f t="shared" si="219"/>
+        <v>172</v>
+      </c>
+      <c r="T397" s="14">
+        <v>0</v>
+      </c>
+      <c r="U397" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="398" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A398" s="7"/>
-      <c r="B398" s="9"/>
-      <c r="C398" s="9"/>
-      <c r="D398" s="9"/>
-      <c r="E398" s="9"/>
-      <c r="F398" s="9"/>
-      <c r="G398" s="9"/>
-      <c r="H398" s="9"/>
-      <c r="I398" s="9"/>
-      <c r="J398" s="9"/>
-      <c r="K398" s="9"/>
-      <c r="L398" s="9"/>
-      <c r="M398" s="9"/>
-      <c r="N398" s="9"/>
-      <c r="O398" s="9"/>
-      <c r="P398" s="12"/>
-      <c r="Q398" s="9"/>
-      <c r="R398" s="9"/>
-      <c r="S398" s="14"/>
-      <c r="T398" s="9"/>
-      <c r="U398" s="14"/>
+      <c r="A398" s="7" t="s">
+        <v>1267</v>
+      </c>
+      <c r="B398" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C398" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D398" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E398" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F398" s="14">
+        <v>246</v>
+      </c>
+      <c r="G398" s="9" t="s">
+        <v>1262</v>
+      </c>
+      <c r="H398" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I398" s="9">
+        <f t="shared" si="224"/>
+        <v>9</v>
+      </c>
+      <c r="J398" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K398" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L398" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M398" s="14">
+        <v>3</v>
+      </c>
+      <c r="N398" s="14">
+        <v>34.99</v>
+      </c>
+      <c r="O398" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P398" s="12" t="s">
+        <v>1268</v>
+      </c>
+      <c r="Q398" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R398" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S398" s="14">
+        <f t="shared" si="219"/>
+        <v>153</v>
+      </c>
+      <c r="T398" s="14">
+        <v>0</v>
+      </c>
+      <c r="U398" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="399" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A399" s="7"/>
-      <c r="B399" s="9"/>
-      <c r="C399" s="9"/>
-      <c r="D399" s="9"/>
-      <c r="E399" s="9"/>
-      <c r="F399" s="9"/>
-      <c r="G399" s="9"/>
-      <c r="H399" s="9"/>
-      <c r="I399" s="9"/>
-      <c r="J399" s="9"/>
-      <c r="K399" s="9"/>
-      <c r="L399" s="9"/>
-      <c r="M399" s="9"/>
-      <c r="N399" s="9"/>
-      <c r="O399" s="9"/>
-      <c r="P399" s="12"/>
-      <c r="Q399" s="9"/>
-      <c r="R399" s="9"/>
-      <c r="S399" s="14"/>
-      <c r="T399" s="9"/>
-      <c r="U399" s="14"/>
+      <c r="A399" s="7" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B399" s="14">
+        <v>2022</v>
+      </c>
+      <c r="C399" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D399" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E399" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F399" s="14">
+        <v>256</v>
+      </c>
+      <c r="G399" s="9" t="s">
+        <v>1270</v>
+      </c>
+      <c r="H399" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I399" s="9">
+        <f t="shared" si="224"/>
+        <v>9</v>
+      </c>
+      <c r="J399" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K399" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L399" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="M399" s="14">
+        <v>2</v>
+      </c>
+      <c r="N399" s="14">
+        <v>39.99</v>
+      </c>
+      <c r="O399" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P399" s="12" t="s">
+        <v>1271</v>
+      </c>
+      <c r="Q399" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R399" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S399" s="14">
+        <f t="shared" si="219"/>
+        <v>72</v>
+      </c>
+      <c r="T399" s="14">
+        <v>0</v>
+      </c>
+      <c r="U399" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="400" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A400" s="7"/>
-      <c r="B400" s="9"/>
-      <c r="C400" s="9"/>
-      <c r="D400" s="9"/>
-      <c r="E400" s="9"/>
-      <c r="F400" s="9"/>
-      <c r="G400" s="9"/>
-      <c r="H400" s="9"/>
-      <c r="I400" s="9"/>
-      <c r="J400" s="9"/>
-      <c r="K400" s="9"/>
-      <c r="L400" s="9"/>
-      <c r="M400" s="9"/>
-      <c r="N400" s="9"/>
-      <c r="O400" s="9"/>
-      <c r="P400" s="12"/>
-      <c r="Q400" s="9"/>
-      <c r="R400" s="9"/>
-      <c r="S400" s="14"/>
-      <c r="T400" s="9"/>
-      <c r="U400" s="14"/>
+      <c r="A400" s="7" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B400" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C400" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D400" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E400" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F400" s="14">
+        <v>458</v>
+      </c>
+      <c r="G400" s="9" t="s">
+        <v>1270</v>
+      </c>
+      <c r="H400" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I400" s="9">
+        <f t="shared" si="224"/>
+        <v>9</v>
+      </c>
+      <c r="J400" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K400" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L400" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="M400" s="14">
+        <v>2</v>
+      </c>
+      <c r="N400" s="14">
+        <v>59.99</v>
+      </c>
+      <c r="O400" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P400" s="12" t="s">
+        <v>1273</v>
+      </c>
+      <c r="Q400" s="9" t="s">
+        <v>538</v>
+      </c>
+      <c r="R400" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S400" s="14">
+        <f t="shared" si="219"/>
+        <v>143</v>
+      </c>
+      <c r="T400" s="14">
+        <v>0</v>
+      </c>
+      <c r="U400" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="401" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A401" s="9"/>

</xml_diff>

<commit_message>
#55 Reading List: updated to 2026-10-04.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE92AB3-44F7-43E6-9B25-AF6B0584C98C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB426F9-566A-40BF-B086-29D56515D5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="735" yWindow="660" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6007" uniqueCount="1274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6031" uniqueCount="1280">
   <si>
     <t>Format</t>
   </si>
@@ -3868,6 +3868,24 @@
   </si>
   <si>
     <t>Useless. Ok as getting started guide, but nothing new for non-beginners. The book is also hyper-dense of examples, which slow down the reading.</t>
+  </si>
+  <si>
+    <t>Spec-Driven Development</t>
+  </si>
+  <si>
+    <t>2026-10-02</t>
+  </si>
+  <si>
+    <t>Useful. Ok to read as an opinion, but very repetitive.</t>
+  </si>
+  <si>
+    <t>Vector Databases: A Practical Introduction</t>
+  </si>
+  <si>
+    <t>2026-10-04</t>
+  </si>
+  <si>
+    <t>Useful. The first part of the book is very concise, clearly explained, with simple examples and easy to scan. The first part captures perfectly the central role of vector databases in the AI world. The second part is just code examples and repetitions.</t>
   </si>
 </sst>
 </file>
@@ -4013,7 +4031,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4134,6 +4152,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -11602,7 +11623,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:U406"/>
+  <dimension ref="A1:U414"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -38066,7 +38087,7 @@
         <v>153</v>
       </c>
       <c r="S389" s="14">
-        <f t="shared" ref="S389:S400" si="219">LEN(P389)</f>
+        <f t="shared" ref="S389:S402" si="219">LEN(P389)</f>
         <v>30</v>
       </c>
       <c r="T389" s="14">
@@ -38371,7 +38392,7 @@
         <v>1258</v>
       </c>
       <c r="H394" s="9">
-        <f t="shared" ref="H394:H400" si="222">YEAR(G394)</f>
+        <f t="shared" ref="H394:H401" si="222">YEAR(G394)</f>
         <v>2026</v>
       </c>
       <c r="I394" s="9">
@@ -38579,7 +38600,7 @@
         <v>2026</v>
       </c>
       <c r="I397" s="9">
-        <f t="shared" ref="I397:I400" si="224">MONTH(G397)</f>
+        <f t="shared" ref="I397:I401" si="224">MONTH(G397)</f>
         <v>9</v>
       </c>
       <c r="J397" s="9" t="s">
@@ -38825,53 +38846,143 @@
       </c>
     </row>
     <row r="401" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A401" s="9"/>
-      <c r="B401" s="9"/>
-      <c r="C401" s="9"/>
-      <c r="D401" s="9"/>
-      <c r="E401" s="9"/>
-      <c r="F401" s="9"/>
-      <c r="G401" s="9"/>
-      <c r="H401" s="9"/>
-      <c r="I401" s="9"/>
-      <c r="J401" s="9"/>
-      <c r="K401" s="9"/>
-      <c r="L401" s="9"/>
-      <c r="M401" s="9"/>
-      <c r="N401" s="9"/>
-      <c r="O401" s="9"/>
-      <c r="P401" s="9"/>
-      <c r="Q401" s="9"/>
-      <c r="R401" s="9"/>
-      <c r="S401" s="14"/>
-      <c r="T401" s="9"/>
-      <c r="U401" s="14"/>
+      <c r="A401" s="7" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B401" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C401" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D401" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E401" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F401" s="44">
+        <v>167</v>
+      </c>
+      <c r="G401" s="9" t="s">
+        <v>1275</v>
+      </c>
+      <c r="H401" s="9">
+        <f t="shared" si="222"/>
+        <v>2026</v>
+      </c>
+      <c r="I401" s="9">
+        <f t="shared" si="224"/>
+        <v>10</v>
+      </c>
+      <c r="J401" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K401" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L401" s="9" t="s">
+        <v>348</v>
+      </c>
+      <c r="M401" s="44">
+        <v>2</v>
+      </c>
+      <c r="N401" s="14">
+        <v>19.989999999999998</v>
+      </c>
+      <c r="O401" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P401" s="7" t="s">
+        <v>1276</v>
+      </c>
+      <c r="Q401" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R401" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S401" s="14">
+        <f t="shared" si="219"/>
+        <v>54</v>
+      </c>
+      <c r="T401" s="14">
+        <v>0</v>
+      </c>
+      <c r="U401" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="402" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A402" s="9"/>
-      <c r="B402" s="9"/>
-      <c r="C402" s="9"/>
-      <c r="D402" s="9"/>
-      <c r="E402" s="9"/>
-      <c r="F402" s="9"/>
-      <c r="G402" s="9"/>
-      <c r="H402" s="9"/>
-      <c r="I402" s="9"/>
-      <c r="J402" s="9"/>
-      <c r="K402" s="9"/>
-      <c r="L402" s="9"/>
-      <c r="M402" s="9"/>
-      <c r="N402" s="9"/>
-      <c r="O402" s="9"/>
-      <c r="P402" s="9"/>
-      <c r="Q402" s="9"/>
-      <c r="R402" s="9"/>
-      <c r="S402" s="14"/>
-      <c r="T402" s="9"/>
-      <c r="U402" s="14"/>
+      <c r="A402" s="7" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B402" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C402" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D402" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E402" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F402" s="44">
+        <v>293</v>
+      </c>
+      <c r="G402" s="9" t="s">
+        <v>1278</v>
+      </c>
+      <c r="H402" s="9">
+        <f t="shared" ref="H402" si="225">YEAR(G402)</f>
+        <v>2026</v>
+      </c>
+      <c r="I402" s="9">
+        <f t="shared" ref="I402" si="226">MONTH(G402)</f>
+        <v>10</v>
+      </c>
+      <c r="J402" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K402" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L402" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M402" s="44">
+        <v>4</v>
+      </c>
+      <c r="N402" s="14">
+        <v>69.989999999999995</v>
+      </c>
+      <c r="O402" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P402" s="7" t="s">
+        <v>1279</v>
+      </c>
+      <c r="Q402" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R402" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S402" s="14">
+        <f t="shared" si="219"/>
+        <v>252</v>
+      </c>
+      <c r="T402" s="14">
+        <v>0</v>
+      </c>
+      <c r="U402" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="403" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A403" s="9"/>
+      <c r="A403" s="7"/>
       <c r="B403" s="9"/>
       <c r="C403" s="9"/>
       <c r="D403" s="9"/>
@@ -38886,7 +38997,7 @@
       <c r="M403" s="9"/>
       <c r="N403" s="9"/>
       <c r="O403" s="9"/>
-      <c r="P403" s="9"/>
+      <c r="P403" s="7"/>
       <c r="Q403" s="9"/>
       <c r="R403" s="9"/>
       <c r="S403" s="14"/>
@@ -38894,7 +39005,7 @@
       <c r="U403" s="14"/>
     </row>
     <row r="404" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A404" s="9"/>
+      <c r="A404" s="7"/>
       <c r="B404" s="9"/>
       <c r="C404" s="9"/>
       <c r="D404" s="9"/>
@@ -38909,7 +39020,7 @@
       <c r="M404" s="9"/>
       <c r="N404" s="9"/>
       <c r="O404" s="9"/>
-      <c r="P404" s="9"/>
+      <c r="P404" s="7"/>
       <c r="Q404" s="9"/>
       <c r="R404" s="9"/>
       <c r="S404" s="14"/>
@@ -38917,7 +39028,7 @@
       <c r="U404" s="14"/>
     </row>
     <row r="405" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A405" s="9"/>
+      <c r="A405" s="7"/>
       <c r="B405" s="9"/>
       <c r="C405" s="9"/>
       <c r="D405" s="9"/>
@@ -38932,7 +39043,7 @@
       <c r="M405" s="9"/>
       <c r="N405" s="9"/>
       <c r="O405" s="9"/>
-      <c r="P405" s="9"/>
+      <c r="P405" s="7"/>
       <c r="Q405" s="9"/>
       <c r="R405" s="9"/>
       <c r="S405" s="14"/>
@@ -38940,7 +39051,7 @@
       <c r="U405" s="14"/>
     </row>
     <row r="406" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A406" s="9"/>
+      <c r="A406" s="7"/>
       <c r="B406" s="9"/>
       <c r="C406" s="9"/>
       <c r="D406" s="9"/>
@@ -38955,12 +39066,196 @@
       <c r="M406" s="9"/>
       <c r="N406" s="9"/>
       <c r="O406" s="9"/>
-      <c r="P406" s="9"/>
+      <c r="P406" s="7"/>
       <c r="Q406" s="9"/>
       <c r="R406" s="9"/>
       <c r="S406" s="14"/>
       <c r="T406" s="9"/>
       <c r="U406" s="14"/>
+    </row>
+    <row r="407" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A407" s="9"/>
+      <c r="B407" s="9"/>
+      <c r="C407" s="9"/>
+      <c r="D407" s="9"/>
+      <c r="E407" s="9"/>
+      <c r="F407" s="9"/>
+      <c r="G407" s="9"/>
+      <c r="H407" s="9"/>
+      <c r="I407" s="9"/>
+      <c r="J407" s="9"/>
+      <c r="K407" s="9"/>
+      <c r="L407" s="9"/>
+      <c r="M407" s="9"/>
+      <c r="N407" s="9"/>
+      <c r="O407" s="9"/>
+      <c r="P407" s="9"/>
+      <c r="Q407" s="9"/>
+      <c r="R407" s="9"/>
+      <c r="S407" s="14"/>
+      <c r="T407" s="9"/>
+      <c r="U407" s="14"/>
+    </row>
+    <row r="408" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A408" s="9"/>
+      <c r="B408" s="9"/>
+      <c r="C408" s="9"/>
+      <c r="D408" s="9"/>
+      <c r="E408" s="9"/>
+      <c r="F408" s="9"/>
+      <c r="G408" s="9"/>
+      <c r="H408" s="9"/>
+      <c r="I408" s="9"/>
+      <c r="J408" s="9"/>
+      <c r="K408" s="9"/>
+      <c r="L408" s="9"/>
+      <c r="M408" s="9"/>
+      <c r="N408" s="9"/>
+      <c r="O408" s="9"/>
+      <c r="P408" s="9"/>
+      <c r="Q408" s="9"/>
+      <c r="R408" s="9"/>
+      <c r="S408" s="14"/>
+      <c r="T408" s="9"/>
+      <c r="U408" s="14"/>
+    </row>
+    <row r="409" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A409" s="9"/>
+      <c r="B409" s="9"/>
+      <c r="C409" s="9"/>
+      <c r="D409" s="9"/>
+      <c r="E409" s="9"/>
+      <c r="F409" s="9"/>
+      <c r="G409" s="9"/>
+      <c r="H409" s="9"/>
+      <c r="I409" s="9"/>
+      <c r="J409" s="9"/>
+      <c r="K409" s="9"/>
+      <c r="L409" s="9"/>
+      <c r="M409" s="9"/>
+      <c r="N409" s="9"/>
+      <c r="O409" s="9"/>
+      <c r="P409" s="9"/>
+      <c r="Q409" s="9"/>
+      <c r="R409" s="9"/>
+      <c r="S409" s="14"/>
+      <c r="T409" s="9"/>
+      <c r="U409" s="14"/>
+    </row>
+    <row r="410" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A410" s="9"/>
+      <c r="B410" s="9"/>
+      <c r="C410" s="9"/>
+      <c r="D410" s="9"/>
+      <c r="E410" s="9"/>
+      <c r="F410" s="9"/>
+      <c r="G410" s="9"/>
+      <c r="H410" s="9"/>
+      <c r="I410" s="9"/>
+      <c r="J410" s="9"/>
+      <c r="K410" s="9"/>
+      <c r="L410" s="9"/>
+      <c r="M410" s="9"/>
+      <c r="N410" s="9"/>
+      <c r="O410" s="9"/>
+      <c r="P410" s="9"/>
+      <c r="Q410" s="9"/>
+      <c r="R410" s="9"/>
+      <c r="S410" s="14"/>
+      <c r="T410" s="9"/>
+      <c r="U410" s="14"/>
+    </row>
+    <row r="411" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A411" s="9"/>
+      <c r="B411" s="9"/>
+      <c r="C411" s="9"/>
+      <c r="D411" s="9"/>
+      <c r="E411" s="9"/>
+      <c r="F411" s="9"/>
+      <c r="G411" s="9"/>
+      <c r="H411" s="9"/>
+      <c r="I411" s="9"/>
+      <c r="J411" s="9"/>
+      <c r="K411" s="9"/>
+      <c r="L411" s="9"/>
+      <c r="M411" s="9"/>
+      <c r="N411" s="9"/>
+      <c r="O411" s="9"/>
+      <c r="P411" s="9"/>
+      <c r="Q411" s="9"/>
+      <c r="R411" s="9"/>
+      <c r="S411" s="14"/>
+      <c r="T411" s="9"/>
+      <c r="U411" s="14"/>
+    </row>
+    <row r="412" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A412" s="9"/>
+      <c r="B412" s="9"/>
+      <c r="C412" s="9"/>
+      <c r="D412" s="9"/>
+      <c r="E412" s="9"/>
+      <c r="F412" s="9"/>
+      <c r="G412" s="9"/>
+      <c r="H412" s="9"/>
+      <c r="I412" s="9"/>
+      <c r="J412" s="9"/>
+      <c r="K412" s="9"/>
+      <c r="L412" s="9"/>
+      <c r="M412" s="9"/>
+      <c r="N412" s="9"/>
+      <c r="O412" s="9"/>
+      <c r="P412" s="9"/>
+      <c r="Q412" s="9"/>
+      <c r="R412" s="9"/>
+      <c r="S412" s="14"/>
+      <c r="T412" s="9"/>
+      <c r="U412" s="14"/>
+    </row>
+    <row r="413" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A413" s="9"/>
+      <c r="B413" s="9"/>
+      <c r="C413" s="9"/>
+      <c r="D413" s="9"/>
+      <c r="E413" s="9"/>
+      <c r="F413" s="9"/>
+      <c r="G413" s="9"/>
+      <c r="H413" s="9"/>
+      <c r="I413" s="9"/>
+      <c r="J413" s="9"/>
+      <c r="K413" s="9"/>
+      <c r="L413" s="9"/>
+      <c r="M413" s="9"/>
+      <c r="N413" s="9"/>
+      <c r="O413" s="9"/>
+      <c r="P413" s="9"/>
+      <c r="Q413" s="9"/>
+      <c r="R413" s="9"/>
+      <c r="S413" s="14"/>
+      <c r="T413" s="9"/>
+      <c r="U413" s="14"/>
+    </row>
+    <row r="414" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A414" s="9"/>
+      <c r="B414" s="9"/>
+      <c r="C414" s="9"/>
+      <c r="D414" s="9"/>
+      <c r="E414" s="9"/>
+      <c r="F414" s="9"/>
+      <c r="G414" s="9"/>
+      <c r="H414" s="9"/>
+      <c r="I414" s="9"/>
+      <c r="J414" s="9"/>
+      <c r="K414" s="9"/>
+      <c r="L414" s="9"/>
+      <c r="M414" s="9"/>
+      <c r="N414" s="9"/>
+      <c r="O414" s="9"/>
+      <c r="P414" s="9"/>
+      <c r="Q414" s="9"/>
+      <c r="R414" s="9"/>
+      <c r="S414" s="14"/>
+      <c r="T414" s="9"/>
+      <c r="U414" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>

<commit_message>
#55 Reading List: updated to 2026-10-17.
</commit_message>
<xml_diff>
--- a/data/Reading List.xlsx
+++ b/data/Reading List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dropbox\Repositories\py-nwreadinglist\nwreadinglist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB426F9-566A-40BF-B086-29D56515D5C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A403FA72-0E89-4C60-9A26-7CAF376990CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="735" yWindow="660" windowWidth="27105" windowHeight="13995" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1635" yWindow="810" windowWidth="23550" windowHeight="13665" tabRatio="313" firstSheet="7" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detailed2016" sheetId="16" state="hidden" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6031" uniqueCount="1280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6127" uniqueCount="1301">
   <si>
     <t>Format</t>
   </si>
@@ -3886,6 +3886,69 @@
   </si>
   <si>
     <t>Useful. The first part of the book is very concise, clearly explained, with simple examples and easy to scan. The first part captures perfectly the central role of vector databases in the AI world. The second part is just code examples and repetitions.</t>
+  </si>
+  <si>
+    <t>The Forward Deployed Engineer</t>
+  </si>
+  <si>
+    <t>2026-10-08</t>
+  </si>
+  <si>
+    <t>Useful. Very redundant, 75 pages could have been summarized in two pages.</t>
+  </si>
+  <si>
+    <t>The OpenClaw Bible</t>
+  </si>
+  <si>
+    <t>Useless. It looks like written by AI. Lot of redundancy, lack of scannable layout.</t>
+  </si>
+  <si>
+    <t>OpenClaw: The Complete Guide</t>
+  </si>
+  <si>
+    <t>2026-10-09</t>
+  </si>
+  <si>
+    <t>Useless. AI-slop book.</t>
+  </si>
+  <si>
+    <t>OpenClaw: The Complete Guide v1.4.0</t>
+  </si>
+  <si>
+    <t>2026-10-15</t>
+  </si>
+  <si>
+    <t>Useful. Ok as getting started guide.</t>
+  </si>
+  <si>
+    <t>The Architect's Paradox</t>
+  </si>
+  <si>
+    <t>Useful. Apart from the very personal parallelism between philosophic concepts throught history and software architecture,  the book is well written and it delivers some useful opinions.</t>
+  </si>
+  <si>
+    <t>Ontological Prisms</t>
+  </si>
+  <si>
+    <t>Useless. The idea behind the book is interesting, but the implementation is awful. The book is extremely redundant and abstract, with no actionable insights for whom works with knowledge management and AI.</t>
+  </si>
+  <si>
+    <t>Generative AI At The Edge</t>
+  </si>
+  <si>
+    <t>2026-10-16</t>
+  </si>
+  <si>
+    <t>Useful. Ok as getting started guide, a bit repetitive in the second half.</t>
+  </si>
+  <si>
+    <t>Harness Engineering (Early Release)</t>
+  </si>
+  <si>
+    <t>2026-10-17</t>
+  </si>
+  <si>
+    <t>Useful. Ok as getting started guide. Code examples should be restructured and proposed in a progressive complexity fashion, instead of being thrown there out-of-the-blue.</t>
   </si>
 </sst>
 </file>
@@ -11623,7 +11686,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:U414"/>
+  <dimension ref="A1:U422"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="57.42578125" style="1" customWidth="1"/>
@@ -38087,7 +38150,7 @@
         <v>153</v>
       </c>
       <c r="S389" s="14">
-        <f t="shared" ref="S389:S402" si="219">LEN(P389)</f>
+        <f t="shared" ref="S389:S401" si="219">LEN(P389)</f>
         <v>30</v>
       </c>
       <c r="T389" s="14">
@@ -38861,7 +38924,7 @@
       <c r="E401" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F401" s="44">
+      <c r="F401" s="14">
         <v>167</v>
       </c>
       <c r="G401" s="9" t="s">
@@ -38884,7 +38947,7 @@
       <c r="L401" s="9" t="s">
         <v>348</v>
       </c>
-      <c r="M401" s="44">
+      <c r="M401" s="14">
         <v>2</v>
       </c>
       <c r="N401" s="14">
@@ -38929,18 +38992,18 @@
       <c r="E402" s="9" t="s">
         <v>634</v>
       </c>
-      <c r="F402" s="44">
+      <c r="F402" s="14">
         <v>293</v>
       </c>
       <c r="G402" s="9" t="s">
         <v>1278</v>
       </c>
       <c r="H402" s="9">
-        <f t="shared" ref="H402" si="225">YEAR(G402)</f>
+        <f t="shared" ref="H402:H403" si="225">YEAR(G402)</f>
         <v>2026</v>
       </c>
       <c r="I402" s="9">
-        <f t="shared" ref="I402" si="226">MONTH(G402)</f>
+        <f t="shared" ref="I402:I403" si="226">MONTH(G402)</f>
         <v>10</v>
       </c>
       <c r="J402" s="9" t="s">
@@ -38952,7 +39015,7 @@
       <c r="L402" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="M402" s="44">
+      <c r="M402" s="14">
         <v>4</v>
       </c>
       <c r="N402" s="14">
@@ -38971,7 +39034,7 @@
         <v>153</v>
       </c>
       <c r="S402" s="14">
-        <f t="shared" si="219"/>
+        <f>LEN(P402)</f>
         <v>252</v>
       </c>
       <c r="T402" s="14">
@@ -38982,191 +39045,551 @@
       </c>
     </row>
     <row r="403" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A403" s="7"/>
-      <c r="B403" s="9"/>
-      <c r="C403" s="9"/>
-      <c r="D403" s="9"/>
-      <c r="E403" s="9"/>
-      <c r="F403" s="9"/>
-      <c r="G403" s="9"/>
-      <c r="H403" s="9"/>
-      <c r="I403" s="9"/>
-      <c r="J403" s="9"/>
-      <c r="K403" s="9"/>
-      <c r="L403" s="9"/>
-      <c r="M403" s="9"/>
-      <c r="N403" s="9"/>
-      <c r="O403" s="9"/>
-      <c r="P403" s="7"/>
-      <c r="Q403" s="9"/>
-      <c r="R403" s="9"/>
-      <c r="S403" s="14"/>
-      <c r="T403" s="9"/>
-      <c r="U403" s="14"/>
+      <c r="A403" s="7" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B403" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C403" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D403" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E403" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F403" s="44">
+        <v>65</v>
+      </c>
+      <c r="G403" s="9" t="s">
+        <v>1281</v>
+      </c>
+      <c r="H403" s="9">
+        <f t="shared" si="225"/>
+        <v>2026</v>
+      </c>
+      <c r="I403" s="9">
+        <f t="shared" si="226"/>
+        <v>10</v>
+      </c>
+      <c r="J403" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K403" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L403" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M403" s="44">
+        <v>2</v>
+      </c>
+      <c r="N403" s="44">
+        <v>49</v>
+      </c>
+      <c r="O403" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P403" s="7" t="s">
+        <v>1282</v>
+      </c>
+      <c r="Q403" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R403" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S403" s="14">
+        <f>LEN(P403)</f>
+        <v>73</v>
+      </c>
+      <c r="T403" s="14">
+        <v>0</v>
+      </c>
+      <c r="U403" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="404" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A404" s="7"/>
-      <c r="B404" s="9"/>
-      <c r="C404" s="9"/>
-      <c r="D404" s="9"/>
-      <c r="E404" s="9"/>
-      <c r="F404" s="9"/>
-      <c r="G404" s="9"/>
-      <c r="H404" s="9"/>
-      <c r="I404" s="9"/>
-      <c r="J404" s="9"/>
-      <c r="K404" s="9"/>
-      <c r="L404" s="9"/>
-      <c r="M404" s="9"/>
-      <c r="N404" s="9"/>
-      <c r="O404" s="9"/>
-      <c r="P404" s="7"/>
-      <c r="Q404" s="9"/>
-      <c r="R404" s="9"/>
-      <c r="S404" s="14"/>
-      <c r="T404" s="9"/>
-      <c r="U404" s="14"/>
+      <c r="A404" s="7" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B404" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C404" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D404" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E404" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F404" s="44">
+        <v>113</v>
+      </c>
+      <c r="G404" s="9" t="s">
+        <v>1281</v>
+      </c>
+      <c r="H404" s="9">
+        <f t="shared" ref="H404" si="227">YEAR(G404)</f>
+        <v>2026</v>
+      </c>
+      <c r="I404" s="9">
+        <f t="shared" ref="I404" si="228">MONTH(G404)</f>
+        <v>10</v>
+      </c>
+      <c r="J404" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K404" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L404" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M404" s="44">
+        <v>1</v>
+      </c>
+      <c r="N404" s="44">
+        <v>14.79</v>
+      </c>
+      <c r="O404" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P404" s="7" t="s">
+        <v>1284</v>
+      </c>
+      <c r="Q404" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R404" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S404" s="14">
+        <f>LEN(P404)</f>
+        <v>82</v>
+      </c>
+      <c r="T404" s="14">
+        <v>0</v>
+      </c>
+      <c r="U404" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="405" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A405" s="7"/>
-      <c r="B405" s="9"/>
-      <c r="C405" s="9"/>
-      <c r="D405" s="9"/>
-      <c r="E405" s="9"/>
-      <c r="F405" s="9"/>
-      <c r="G405" s="9"/>
-      <c r="H405" s="9"/>
-      <c r="I405" s="9"/>
-      <c r="J405" s="9"/>
-      <c r="K405" s="9"/>
-      <c r="L405" s="9"/>
-      <c r="M405" s="9"/>
-      <c r="N405" s="9"/>
-      <c r="O405" s="9"/>
-      <c r="P405" s="7"/>
-      <c r="Q405" s="9"/>
-      <c r="R405" s="9"/>
-      <c r="S405" s="14"/>
-      <c r="T405" s="9"/>
-      <c r="U405" s="14"/>
+      <c r="A405" s="7" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B405" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C405" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D405" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E405" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F405" s="44">
+        <v>51</v>
+      </c>
+      <c r="G405" s="9" t="s">
+        <v>1286</v>
+      </c>
+      <c r="H405" s="9">
+        <f t="shared" ref="H405" si="229">YEAR(G405)</f>
+        <v>2026</v>
+      </c>
+      <c r="I405" s="9">
+        <f t="shared" ref="I405" si="230">MONTH(G405)</f>
+        <v>10</v>
+      </c>
+      <c r="J405" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K405" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L405" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M405" s="44">
+        <v>1</v>
+      </c>
+      <c r="N405" s="44">
+        <v>0</v>
+      </c>
+      <c r="O405" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P405" s="7" t="s">
+        <v>1287</v>
+      </c>
+      <c r="Q405" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R405" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S405" s="14">
+        <f>LEN(P405)</f>
+        <v>22</v>
+      </c>
+      <c r="T405" s="14">
+        <v>0</v>
+      </c>
+      <c r="U405" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="406" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A406" s="7"/>
-      <c r="B406" s="9"/>
-      <c r="C406" s="9"/>
-      <c r="D406" s="9"/>
-      <c r="E406" s="9"/>
-      <c r="F406" s="9"/>
-      <c r="G406" s="9"/>
-      <c r="H406" s="9"/>
-      <c r="I406" s="9"/>
-      <c r="J406" s="9"/>
-      <c r="K406" s="9"/>
-      <c r="L406" s="9"/>
-      <c r="M406" s="9"/>
-      <c r="N406" s="9"/>
-      <c r="O406" s="9"/>
-      <c r="P406" s="7"/>
-      <c r="Q406" s="9"/>
-      <c r="R406" s="9"/>
-      <c r="S406" s="14"/>
-      <c r="T406" s="9"/>
-      <c r="U406" s="14"/>
+      <c r="A406" s="7" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B406" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C406" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D406" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E406" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F406" s="44">
+        <v>110</v>
+      </c>
+      <c r="G406" s="9" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H406" s="9">
+        <f t="shared" ref="H406" si="231">YEAR(G406)</f>
+        <v>2026</v>
+      </c>
+      <c r="I406" s="9">
+        <f t="shared" ref="I406" si="232">MONTH(G406)</f>
+        <v>10</v>
+      </c>
+      <c r="J406" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K406" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L406" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M406" s="44">
+        <v>3</v>
+      </c>
+      <c r="N406" s="44">
+        <v>0</v>
+      </c>
+      <c r="O406" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P406" s="7" t="s">
+        <v>1290</v>
+      </c>
+      <c r="Q406" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R406" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S406" s="14">
+        <f>LEN(P406)</f>
+        <v>36</v>
+      </c>
+      <c r="T406" s="14">
+        <v>0</v>
+      </c>
+      <c r="U406" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="407" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A407" s="9"/>
-      <c r="B407" s="9"/>
-      <c r="C407" s="9"/>
-      <c r="D407" s="9"/>
-      <c r="E407" s="9"/>
-      <c r="F407" s="9"/>
-      <c r="G407" s="9"/>
-      <c r="H407" s="9"/>
-      <c r="I407" s="9"/>
-      <c r="J407" s="9"/>
-      <c r="K407" s="9"/>
-      <c r="L407" s="9"/>
-      <c r="M407" s="9"/>
-      <c r="N407" s="9"/>
-      <c r="O407" s="9"/>
-      <c r="P407" s="9"/>
-      <c r="Q407" s="9"/>
-      <c r="R407" s="9"/>
-      <c r="S407" s="14"/>
-      <c r="T407" s="9"/>
-      <c r="U407" s="14"/>
+      <c r="A407" s="7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B407" s="14">
+        <v>2025</v>
+      </c>
+      <c r="C407" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D407" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E407" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F407" s="44">
+        <v>171</v>
+      </c>
+      <c r="G407" s="9" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H407" s="9">
+        <f t="shared" ref="H407" si="233">YEAR(G407)</f>
+        <v>2026</v>
+      </c>
+      <c r="I407" s="9">
+        <f t="shared" ref="I407" si="234">MONTH(G407)</f>
+        <v>10</v>
+      </c>
+      <c r="J407" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K407" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L407" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M407" s="44">
+        <v>3</v>
+      </c>
+      <c r="N407" s="44">
+        <v>25</v>
+      </c>
+      <c r="O407" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P407" s="12" t="s">
+        <v>1292</v>
+      </c>
+      <c r="Q407" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R407" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S407" s="14">
+        <f>LEN(P407)</f>
+        <v>185</v>
+      </c>
+      <c r="T407" s="14">
+        <v>0</v>
+      </c>
+      <c r="U407" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="408" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A408" s="9"/>
-      <c r="B408" s="9"/>
-      <c r="C408" s="9"/>
-      <c r="D408" s="9"/>
-      <c r="E408" s="9"/>
-      <c r="F408" s="9"/>
-      <c r="G408" s="9"/>
-      <c r="H408" s="9"/>
-      <c r="I408" s="9"/>
-      <c r="J408" s="9"/>
-      <c r="K408" s="9"/>
-      <c r="L408" s="9"/>
-      <c r="M408" s="9"/>
-      <c r="N408" s="9"/>
-      <c r="O408" s="9"/>
-      <c r="P408" s="9"/>
-      <c r="Q408" s="9"/>
-      <c r="R408" s="9"/>
-      <c r="S408" s="14"/>
-      <c r="T408" s="9"/>
-      <c r="U408" s="14"/>
+      <c r="A408" s="7" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B408" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C408" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D408" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E408" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F408" s="44">
+        <v>349</v>
+      </c>
+      <c r="G408" s="9" t="s">
+        <v>1289</v>
+      </c>
+      <c r="H408" s="9">
+        <f t="shared" ref="H408" si="235">YEAR(G408)</f>
+        <v>2026</v>
+      </c>
+      <c r="I408" s="9">
+        <f t="shared" ref="I408" si="236">MONTH(G408)</f>
+        <v>10</v>
+      </c>
+      <c r="J408" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K408" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L408" s="9" t="s">
+        <v>352</v>
+      </c>
+      <c r="M408" s="44">
+        <v>1</v>
+      </c>
+      <c r="N408" s="44">
+        <v>145</v>
+      </c>
+      <c r="O408" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P408" s="12" t="s">
+        <v>1294</v>
+      </c>
+      <c r="Q408" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="R408" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S408" s="14">
+        <f>LEN(P408)</f>
+        <v>205</v>
+      </c>
+      <c r="T408" s="14">
+        <v>0</v>
+      </c>
+      <c r="U408" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="409" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A409" s="9"/>
-      <c r="B409" s="9"/>
-      <c r="C409" s="9"/>
-      <c r="D409" s="9"/>
-      <c r="E409" s="9"/>
-      <c r="F409" s="9"/>
-      <c r="G409" s="9"/>
-      <c r="H409" s="9"/>
-      <c r="I409" s="9"/>
-      <c r="J409" s="9"/>
-      <c r="K409" s="9"/>
-      <c r="L409" s="9"/>
-      <c r="M409" s="9"/>
-      <c r="N409" s="9"/>
-      <c r="O409" s="9"/>
-      <c r="P409" s="9"/>
-      <c r="Q409" s="9"/>
-      <c r="R409" s="9"/>
-      <c r="S409" s="14"/>
-      <c r="T409" s="9"/>
-      <c r="U409" s="14"/>
+      <c r="A409" s="7" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B409" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C409" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D409" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E409" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F409" s="44">
+        <v>383</v>
+      </c>
+      <c r="G409" s="9" t="s">
+        <v>1296</v>
+      </c>
+      <c r="H409" s="9">
+        <f t="shared" ref="H409" si="237">YEAR(G409)</f>
+        <v>2026</v>
+      </c>
+      <c r="I409" s="9">
+        <f t="shared" ref="I409" si="238">MONTH(G409)</f>
+        <v>10</v>
+      </c>
+      <c r="J409" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K409" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L409" s="9" t="s">
+        <v>570</v>
+      </c>
+      <c r="M409" s="44">
+        <v>2</v>
+      </c>
+      <c r="N409" s="44">
+        <v>0</v>
+      </c>
+      <c r="O409" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P409" s="7" t="s">
+        <v>1297</v>
+      </c>
+      <c r="Q409" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R409" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S409" s="14">
+        <f>LEN(P409)</f>
+        <v>73</v>
+      </c>
+      <c r="T409" s="14">
+        <v>0</v>
+      </c>
+      <c r="U409" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="410" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A410" s="9"/>
-      <c r="B410" s="9"/>
-      <c r="C410" s="9"/>
-      <c r="D410" s="9"/>
-      <c r="E410" s="9"/>
-      <c r="F410" s="9"/>
-      <c r="G410" s="9"/>
-      <c r="H410" s="9"/>
-      <c r="I410" s="9"/>
-      <c r="J410" s="9"/>
-      <c r="K410" s="9"/>
-      <c r="L410" s="9"/>
-      <c r="M410" s="9"/>
-      <c r="N410" s="9"/>
-      <c r="O410" s="9"/>
-      <c r="P410" s="9"/>
-      <c r="Q410" s="9"/>
-      <c r="R410" s="9"/>
-      <c r="S410" s="14"/>
-      <c r="T410" s="9"/>
-      <c r="U410" s="14"/>
+      <c r="A410" s="7" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B410" s="14">
+        <v>2026</v>
+      </c>
+      <c r="C410" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D410" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E410" s="9" t="s">
+        <v>634</v>
+      </c>
+      <c r="F410" s="44">
+        <v>75</v>
+      </c>
+      <c r="G410" s="9" t="s">
+        <v>1299</v>
+      </c>
+      <c r="H410" s="9">
+        <f t="shared" ref="H410" si="239">YEAR(G410)</f>
+        <v>2026</v>
+      </c>
+      <c r="I410" s="9">
+        <f t="shared" ref="I410" si="240">MONTH(G410)</f>
+        <v>10</v>
+      </c>
+      <c r="J410" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="K410" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="L410" s="9" t="s">
+        <v>343</v>
+      </c>
+      <c r="M410" s="44">
+        <v>3</v>
+      </c>
+      <c r="N410" s="44">
+        <v>49</v>
+      </c>
+      <c r="O410" s="9" t="s">
+        <v>632</v>
+      </c>
+      <c r="P410" s="7" t="s">
+        <v>1300</v>
+      </c>
+      <c r="Q410" s="9" t="s">
+        <v>919</v>
+      </c>
+      <c r="R410" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="S410" s="14">
+        <f>LEN(P410)</f>
+        <v>170</v>
+      </c>
+      <c r="T410" s="14">
+        <v>0</v>
+      </c>
+      <c r="U410" s="14">
+        <v>0</v>
+      </c>
     </row>
     <row r="411" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A411" s="9"/>
+      <c r="A411" s="7"/>
       <c r="B411" s="9"/>
       <c r="C411" s="9"/>
       <c r="D411" s="9"/>
@@ -39181,7 +39604,7 @@
       <c r="M411" s="9"/>
       <c r="N411" s="9"/>
       <c r="O411" s="9"/>
-      <c r="P411" s="9"/>
+      <c r="P411" s="7"/>
       <c r="Q411" s="9"/>
       <c r="R411" s="9"/>
       <c r="S411" s="14"/>
@@ -39189,7 +39612,7 @@
       <c r="U411" s="14"/>
     </row>
     <row r="412" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A412" s="9"/>
+      <c r="A412" s="7"/>
       <c r="B412" s="9"/>
       <c r="C412" s="9"/>
       <c r="D412" s="9"/>
@@ -39204,7 +39627,7 @@
       <c r="M412" s="9"/>
       <c r="N412" s="9"/>
       <c r="O412" s="9"/>
-      <c r="P412" s="9"/>
+      <c r="P412" s="7"/>
       <c r="Q412" s="9"/>
       <c r="R412" s="9"/>
       <c r="S412" s="14"/>
@@ -39212,7 +39635,7 @@
       <c r="U412" s="14"/>
     </row>
     <row r="413" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A413" s="9"/>
+      <c r="A413" s="7"/>
       <c r="B413" s="9"/>
       <c r="C413" s="9"/>
       <c r="D413" s="9"/>
@@ -39227,7 +39650,7 @@
       <c r="M413" s="9"/>
       <c r="N413" s="9"/>
       <c r="O413" s="9"/>
-      <c r="P413" s="9"/>
+      <c r="P413" s="7"/>
       <c r="Q413" s="9"/>
       <c r="R413" s="9"/>
       <c r="S413" s="14"/>
@@ -39235,7 +39658,7 @@
       <c r="U413" s="14"/>
     </row>
     <row r="414" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A414" s="9"/>
+      <c r="A414" s="7"/>
       <c r="B414" s="9"/>
       <c r="C414" s="9"/>
       <c r="D414" s="9"/>
@@ -39250,12 +39673,196 @@
       <c r="M414" s="9"/>
       <c r="N414" s="9"/>
       <c r="O414" s="9"/>
-      <c r="P414" s="9"/>
+      <c r="P414" s="7"/>
       <c r="Q414" s="9"/>
       <c r="R414" s="9"/>
       <c r="S414" s="14"/>
       <c r="T414" s="9"/>
       <c r="U414" s="14"/>
+    </row>
+    <row r="415" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A415" s="7"/>
+      <c r="B415" s="9"/>
+      <c r="C415" s="9"/>
+      <c r="D415" s="9"/>
+      <c r="E415" s="9"/>
+      <c r="F415" s="9"/>
+      <c r="G415" s="9"/>
+      <c r="H415" s="9"/>
+      <c r="I415" s="9"/>
+      <c r="J415" s="9"/>
+      <c r="K415" s="9"/>
+      <c r="L415" s="9"/>
+      <c r="M415" s="9"/>
+      <c r="N415" s="9"/>
+      <c r="O415" s="9"/>
+      <c r="P415" s="7"/>
+      <c r="Q415" s="9"/>
+      <c r="R415" s="9"/>
+      <c r="S415" s="14"/>
+      <c r="T415" s="9"/>
+      <c r="U415" s="14"/>
+    </row>
+    <row r="416" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A416" s="7"/>
+      <c r="B416" s="9"/>
+      <c r="C416" s="9"/>
+      <c r="D416" s="9"/>
+      <c r="E416" s="9"/>
+      <c r="F416" s="9"/>
+      <c r="G416" s="9"/>
+      <c r="H416" s="9"/>
+      <c r="I416" s="9"/>
+      <c r="J416" s="9"/>
+      <c r="K416" s="9"/>
+      <c r="L416" s="9"/>
+      <c r="M416" s="9"/>
+      <c r="N416" s="9"/>
+      <c r="O416" s="9"/>
+      <c r="P416" s="7"/>
+      <c r="Q416" s="9"/>
+      <c r="R416" s="9"/>
+      <c r="S416" s="14"/>
+      <c r="T416" s="9"/>
+      <c r="U416" s="14"/>
+    </row>
+    <row r="417" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A417" s="7"/>
+      <c r="B417" s="9"/>
+      <c r="C417" s="9"/>
+      <c r="D417" s="9"/>
+      <c r="E417" s="9"/>
+      <c r="F417" s="9"/>
+      <c r="G417" s="9"/>
+      <c r="H417" s="9"/>
+      <c r="I417" s="9"/>
+      <c r="J417" s="9"/>
+      <c r="K417" s="9"/>
+      <c r="L417" s="9"/>
+      <c r="M417" s="9"/>
+      <c r="N417" s="9"/>
+      <c r="O417" s="9"/>
+      <c r="P417" s="7"/>
+      <c r="Q417" s="9"/>
+      <c r="R417" s="9"/>
+      <c r="S417" s="14"/>
+      <c r="T417" s="9"/>
+      <c r="U417" s="14"/>
+    </row>
+    <row r="418" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A418" s="7"/>
+      <c r="B418" s="9"/>
+      <c r="C418" s="9"/>
+      <c r="D418" s="9"/>
+      <c r="E418" s="9"/>
+      <c r="F418" s="9"/>
+      <c r="G418" s="9"/>
+      <c r="H418" s="9"/>
+      <c r="I418" s="9"/>
+      <c r="J418" s="9"/>
+      <c r="K418" s="9"/>
+      <c r="L418" s="9"/>
+      <c r="M418" s="9"/>
+      <c r="N418" s="9"/>
+      <c r="O418" s="9"/>
+      <c r="P418" s="7"/>
+      <c r="Q418" s="9"/>
+      <c r="R418" s="9"/>
+      <c r="S418" s="14"/>
+      <c r="T418" s="9"/>
+      <c r="U418" s="14"/>
+    </row>
+    <row r="419" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A419" s="7"/>
+      <c r="B419" s="9"/>
+      <c r="C419" s="9"/>
+      <c r="D419" s="9"/>
+      <c r="E419" s="9"/>
+      <c r="F419" s="9"/>
+      <c r="G419" s="9"/>
+      <c r="H419" s="9"/>
+      <c r="I419" s="9"/>
+      <c r="J419" s="9"/>
+      <c r="K419" s="9"/>
+      <c r="L419" s="9"/>
+      <c r="M419" s="9"/>
+      <c r="N419" s="9"/>
+      <c r="O419" s="9"/>
+      <c r="P419" s="7"/>
+      <c r="Q419" s="9"/>
+      <c r="R419" s="9"/>
+      <c r="S419" s="14"/>
+      <c r="T419" s="9"/>
+      <c r="U419" s="14"/>
+    </row>
+    <row r="420" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A420" s="7"/>
+      <c r="B420" s="9"/>
+      <c r="C420" s="9"/>
+      <c r="D420" s="9"/>
+      <c r="E420" s="9"/>
+      <c r="F420" s="9"/>
+      <c r="G420" s="9"/>
+      <c r="H420" s="9"/>
+      <c r="I420" s="9"/>
+      <c r="J420" s="9"/>
+      <c r="K420" s="9"/>
+      <c r="L420" s="9"/>
+      <c r="M420" s="9"/>
+      <c r="N420" s="9"/>
+      <c r="O420" s="9"/>
+      <c r="P420" s="7"/>
+      <c r="Q420" s="9"/>
+      <c r="R420" s="9"/>
+      <c r="S420" s="14"/>
+      <c r="T420" s="9"/>
+      <c r="U420" s="14"/>
+    </row>
+    <row r="421" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A421" s="7"/>
+      <c r="B421" s="9"/>
+      <c r="C421" s="9"/>
+      <c r="D421" s="9"/>
+      <c r="E421" s="9"/>
+      <c r="F421" s="9"/>
+      <c r="G421" s="9"/>
+      <c r="H421" s="9"/>
+      <c r="I421" s="9"/>
+      <c r="J421" s="9"/>
+      <c r="K421" s="9"/>
+      <c r="L421" s="9"/>
+      <c r="M421" s="9"/>
+      <c r="N421" s="9"/>
+      <c r="O421" s="9"/>
+      <c r="P421" s="7"/>
+      <c r="Q421" s="9"/>
+      <c r="R421" s="9"/>
+      <c r="S421" s="14"/>
+      <c r="T421" s="9"/>
+      <c r="U421" s="14"/>
+    </row>
+    <row r="422" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="A422" s="7"/>
+      <c r="B422" s="9"/>
+      <c r="C422" s="9"/>
+      <c r="D422" s="9"/>
+      <c r="E422" s="9"/>
+      <c r="F422" s="9"/>
+      <c r="G422" s="9"/>
+      <c r="H422" s="9"/>
+      <c r="I422" s="9"/>
+      <c r="J422" s="9"/>
+      <c r="K422" s="9"/>
+      <c r="L422" s="9"/>
+      <c r="M422" s="9"/>
+      <c r="N422" s="9"/>
+      <c r="O422" s="9"/>
+      <c r="P422" s="7"/>
+      <c r="Q422" s="9"/>
+      <c r="R422" s="9"/>
+      <c r="S422" s="14"/>
+      <c r="T422" s="9"/>
+      <c r="U422" s="14"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>